<commit_message>
chore: overwrite 月報表.xlsx via Streamlit restore
</commit_message>
<xml_diff>
--- a/data/月報表.xlsx
+++ b/data/月報表.xlsx
@@ -413,19 +413,211 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>DiscountPolicy</t>
+          <t>年份</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>MonthKey</t>
-        </is>
+          <t>月份</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>營業額</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>商品成本</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>折扣優惠</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>手續費</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>未取貨/退貨運費</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>物流處理費（運費差額）</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>其他費用（一）</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>其他費用（二）</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>薪資費用</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>委製費用</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>蝦皮廣告費用</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>露天廣告費用</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>MO店廣告費用</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>官網廣告費用</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>其他廣告費用</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>耗材費用</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>營業稅額</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>官網月費</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>會計記帳費</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>會費＆勞健保費</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>廣告費用合計</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>總成本</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>淨利</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1091288</v>
+      </c>
+      <c r="D2" t="n">
+        <v>477085</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16005</v>
+      </c>
+      <c r="F2" t="n">
+        <v>158083</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1808</v>
+      </c>
+      <c r="H2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>48729</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4950</v>
+      </c>
+      <c r="M2" t="n">
+        <v>144651</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>8265</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1231</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1900</v>
+      </c>
+      <c r="V2" t="n">
+        <v>4107</v>
+      </c>
+      <c r="W2" t="n">
+        <v>149651</v>
+      </c>
+      <c r="X2" t="n">
+        <v>879074</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>212214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>